<commit_message>
fix(calculators): made method 2 EF calculate on N rate & moved area input
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/5.1-inorganic-fertiliser.xlsx
+++ b/packages/calculators/src/modules/test/5.1-inorganic-fertiliser.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2009B18-BAE1-154B-A813-6ECEE66B5086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB291A4E-9E74-0E4D-BC93-C7D756A8F630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15980" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
   <sheets>
     <sheet name="5.1.1.1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="58">
   <si>
     <t>MNjf</t>
   </si>
@@ -197,9 +197,6 @@
     </r>
   </si>
   <si>
-    <t>Fnorganicf</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
@@ -209,12 +206,6 @@
     <t>Method 1</t>
   </si>
   <si>
-    <t>Table A.2.2.6</t>
-  </si>
-  <si>
-    <t>Custom Fnorganicf</t>
-  </si>
-  <si>
     <t>Urea</t>
   </si>
   <si>
@@ -456,18 +447,6 @@
     <t>Total mass applied (kg)</t>
   </si>
   <si>
-    <t>𝐸𝐹𝑓𝑗=𝑛𝑜𝑛𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑔𝑟𝑎𝑖𝑛𝑠,𝑁2𝑂 = (0.0781 + (0.0075 × 𝑁𝑓𝑗=𝑛𝑜𝑛𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑔𝑟𝑎𝑖𝑛𝑠)) × 10−2</t>
-  </si>
-  <si>
-    <t>𝐸𝐹𝑓𝑗=𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑚𝑎𝑖𝑧𝑒,𝑁2𝑂 = (−0.1474 + (0.0061 × 𝑁𝑓𝑗=𝑖𝑟𝑟𝑖𝑔𝑎𝑡𝑒𝑑𝑚𝑎𝑖𝑧𝑒 )) × 10−2</t>
-  </si>
-  <si>
-    <t>(0.29 + (0.007(𝑒^0.037×𝑁𝑓𝑗=𝑐𝑜𝑡𝑡𝑜𝑛 − 1)) / 𝑁𝑓𝑗=𝑐𝑜𝑡𝑡𝑜𝑛) × 10−2 (Capped at 0.0183)</t>
-  </si>
-  <si>
-    <t>NOTE: I've removed the '0.01' term from below because I believe it is a mistake, confirmation of this is still pending.</t>
-  </si>
-  <si>
     <t>Application rate (kg / hectare)</t>
   </si>
   <si>
@@ -480,13 +459,25 @@
     <t>Application area</t>
   </si>
   <si>
-    <t>Method 2 maize</t>
-  </si>
-  <si>
-    <t>Method 2 grains</t>
-  </si>
-  <si>
-    <t>Method 2 cotton</t>
+    <t>Table A.2.2.1</t>
+  </si>
+  <si>
+    <t>Nfj</t>
+  </si>
+  <si>
+    <t>FNinorganicf</t>
+  </si>
+  <si>
+    <t>Custom FNinorganicf</t>
+  </si>
+  <si>
+    <t>Ammonium Sulfate</t>
+  </si>
+  <si>
+    <t>Calcium Nitrate</t>
+  </si>
+  <si>
+    <t>Method 2 - individual test cases</t>
   </si>
 </sst>
 </file>
@@ -955,7 +946,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78A5655F-5BFE-554E-A3D3-9DFA9517010F}">
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:R35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="17.33203125" style="3" customWidth="1"/>
@@ -966,9 +957,9 @@
     <col min="15" max="15" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="17">
+    <row r="1" spans="1:18" ht="17">
       <c r="A1" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>6</v>
@@ -977,34 +968,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:18">
       <c r="E2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="J2" s="1"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:16" ht="17">
+    <row r="3" spans="1:18" ht="17">
       <c r="A3" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>5</v>
       </c>
       <c r="F3" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>12</v>
+        <v>54</v>
+      </c>
+      <c r="H3" t="s">
+        <v>52</v>
       </c>
       <c r="J3" t="s">
         <v>0</v>
@@ -1019,15 +1013,15 @@
         <v>4</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="17">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="17">
       <c r="A4" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E4">
         <v>50</v>
@@ -1060,22 +1054,22 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="17">
+    <row r="5" spans="1:18" ht="17">
       <c r="A5" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E5">
         <v>40</v>
       </c>
       <c r="F5">
-        <f t="shared" ref="F5:F19" si="0">IF(ISBLANK(B5), "", VLOOKUP(B5,$O$24:$P$30, 2, FALSE))</f>
+        <f>IF(ISBLANK(B5), "", VLOOKUP(B5,$O$24:$P$30, 2, FALSE))</f>
         <v>0.18</v>
       </c>
       <c r="J5">
-        <f t="shared" ref="J5:J24" si="1">IF(ISBLANK(B5), "", IF(ISNUMBER(G5), G5*E5, F5*E5))</f>
+        <f t="shared" ref="J5:J10" si="0">IF(ISBLANK(B5), "", IF(ISNUMBER(G5), G5*E5, F5*E5))</f>
         <v>7.1999999999999993</v>
       </c>
       <c r="K5">
@@ -1091,26 +1085,26 @@
         <v>6.6693599999999994E-5</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:18">
       <c r="A6" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2"/>
       <c r="E6">
         <v>30</v>
       </c>
       <c r="F6">
-        <f t="shared" si="0"/>
+        <f>IF(ISBLANK(B6), "", VLOOKUP(B6,$O$24:$P$30, 2, FALSE))</f>
         <v>0.21</v>
       </c>
       <c r="G6">
         <v>0.25</v>
       </c>
       <c r="J6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>7.5</v>
       </c>
       <c r="K6">
@@ -1126,233 +1120,314 @@
         <v>3.0614999999999997E-5</v>
       </c>
       <c r="O6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18">
       <c r="F7" t="str">
+        <f>IF(ISBLANK(B7), "", VLOOKUP(B7,$O$24:$P$30, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J7" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
       <c r="L7" t="str">
-        <f t="shared" ref="L7:L18" si="2">IF(ISBLANK(K7), "",$P$4)</f>
+        <f t="shared" ref="L7:L10" si="1">IF(ISBLANK(K7), "",$P$4)</f>
         <v/>
       </c>
       <c r="M7" t="str">
-        <f t="shared" ref="M7:M18" si="3">IF(ISBLANK(A7), "", J7*K7*L7/1000)</f>
+        <f>IF(ISBLANK(A7), "", J7*K7*L7/1000)</f>
         <v/>
       </c>
       <c r="O7" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="P7" s="2">
         <v>5.8999999999999999E-3</v>
       </c>
-    </row>
-    <row r="8" spans="1:16">
+      <c r="R7" s="2"/>
+    </row>
+    <row r="8" spans="1:18">
       <c r="F8" t="str">
+        <f>IF(ISBLANK(B8), "", VLOOKUP(B8,$O$24:$P$30, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="J8" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J8" t="str">
+      <c r="L8" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L8" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
       <c r="M8" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(A8), "", J8*K8*L8/1000)</f>
         <v/>
       </c>
       <c r="O8" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P8" s="2">
         <v>7.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" ht="17">
+      <c r="R8" s="2"/>
+    </row>
+    <row r="9" spans="1:18" ht="51">
       <c r="A9" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F9" t="str">
+        <f>IF(ISBLANK(B9), "", VLOOKUP(B9,$O$24:$P$30, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="K9" s="1"/>
       <c r="O9" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="P9" s="2">
         <v>1.8E-3</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" ht="34">
+      <c r="R9" s="2"/>
+    </row>
+    <row r="10" spans="1:18" ht="34">
       <c r="A10" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C10" s="2">
-        <f>175</f>
-        <v>175</v>
+        <v>10</v>
       </c>
       <c r="D10">
         <f>E10/C10</f>
-        <v>40</v>
+        <v>700</v>
       </c>
       <c r="E10">
         <v>7000</v>
       </c>
       <c r="F10">
+        <f t="shared" ref="F10:F11" si="2">IF(ISBLANK(B10), "", VLOOKUP(B10,$O$24:$P$32, 2, FALSE))</f>
+        <v>0.21</v>
+      </c>
+      <c r="H10">
+        <f>D10*IF(G10&lt;&gt;"", G10, F10)</f>
+        <v>147</v>
+      </c>
+      <c r="J10">
         <f t="shared" si="0"/>
-        <v>0.21</v>
-      </c>
-      <c r="J10">
+        <v>1470</v>
+      </c>
+      <c r="K10">
+        <f>MAX(_xlfn.IFS(A10="Irrigated crop (maize)", (-0.1474 + (0.0061 * H10)) * 10^-2, A10="Non-irrigated crop (high rainfall)", (0.0781 + (0.0075*H10)) * 10^-2, A10="Cotton", ((0.29 + (0.007*(EXP(0.037*MIN(H10, 300)) - 1)/MIN(H10, 300))) * 10^-2)), 0)</f>
+        <v>7.4930000000000005E-3</v>
+      </c>
+      <c r="L10">
         <f t="shared" si="1"/>
-        <v>1470</v>
-      </c>
-      <c r="K10">
-        <f>(-0.1474 + (0.0061 * D10)) * 10^-2</f>
-        <v>9.6600000000000017E-4</v>
-      </c>
-      <c r="L10">
-        <f t="shared" si="2"/>
         <v>1.57</v>
       </c>
       <c r="M10" s="5">
         <f>IF(ISBLANK(A10), "", J10*K10*L10/1000)</f>
-        <v>2.2294314000000006E-3</v>
+        <v>1.7293094700000001E-2</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="P10" s="2">
         <v>2.8999999999999998E-3</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" ht="34">
+      <c r="R10" s="2"/>
+    </row>
+    <row r="11" spans="1:18" ht="34">
       <c r="A11" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C11">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="D11">
         <f>E11/C11</f>
-        <v>35.294117647058826</v>
+        <v>300</v>
       </c>
       <c r="E11">
         <v>3000</v>
       </c>
       <c r="F11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0.46</v>
       </c>
       <c r="G11">
         <v>0.4</v>
       </c>
+      <c r="H11">
+        <f>D11*IF(G11&lt;&gt;"", G11, F11)</f>
+        <v>120</v>
+      </c>
       <c r="J11">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B11), "", IF(ISNUMBER(G11), G11*E11, F11*E11))</f>
         <v>1200</v>
       </c>
       <c r="K11">
-        <f>(-0.1474 + (0.0061 * D11)) * 10^-2</f>
-        <v>6.7894117647058854E-4</v>
+        <f t="shared" ref="K11:K19" si="3">MAX(_xlfn.IFS(A11="Irrigated crop (maize)", (-0.1474 + (0.0061 * H11)) * 10^-2, A11="Non-irrigated crop (high rainfall)", (0.0781 + (0.0075*H11)) * 10^-2, A11="Cotton", ((0.29 + (0.007*(EXP(0.037*MIN(H11, 300)) - 1)/MIN(H11, 300))) * 10^-2)), 0)</f>
+        <v>5.8460000000000014E-3</v>
       </c>
       <c r="L11">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(K11), "",$P$4)</f>
         <v>1.57</v>
       </c>
       <c r="M11" s="5">
-        <f t="shared" ref="M11" si="4">IF(ISBLANK(A11), "", J11*K11*L11/1000)</f>
-        <v>1.2791251764705889E-3</v>
+        <f>IF(ISBLANK(A11), "", J11*K11*L11/1000)</f>
+        <v>1.1013864000000003E-2</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="P11" s="2">
         <v>8.0000000000000002E-3</v>
       </c>
-    </row>
-    <row r="12" spans="1:16">
-      <c r="J12" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="R11" s="2"/>
+    </row>
+    <row r="12" spans="1:18" ht="34">
+      <c r="A12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12">
+        <v>10</v>
+      </c>
+      <c r="D12">
+        <f>E12/C12</f>
+        <v>300</v>
+      </c>
+      <c r="E12">
+        <v>3000</v>
+      </c>
+      <c r="F12">
+        <f>IF(ISBLANK(B12), "", VLOOKUP(B12,$O$24:$P$32, 2, FALSE))</f>
+        <v>0.1</v>
+      </c>
+      <c r="H12">
+        <f>D12*IF(G12&lt;&gt;"", G12, F12)</f>
+        <v>30</v>
+      </c>
+      <c r="J12">
+        <f>IF(ISBLANK(B12), "", IF(ISNUMBER(G12), G12*E12, F12*E12))</f>
+        <v>300</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="3"/>
+        <v>3.560000000000002E-4</v>
+      </c>
+      <c r="L12">
+        <f>IF(ISBLANK(K12), "",$P$4)</f>
+        <v>1.57</v>
+      </c>
+      <c r="M12" s="5">
+        <f>IF(ISBLANK(A12), "", J12*K12*L12/1000)</f>
+        <v>1.6767600000000009E-4</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="P12" s="2">
         <v>1.9900000000000001E-2</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" ht="17">
-      <c r="A13" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="F13" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>50</v>
+      <c r="R12" s="2"/>
+    </row>
+    <row r="13" spans="1:18" ht="34">
+      <c r="A13" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="2">
+        <v>10</v>
+      </c>
+      <c r="D13">
+        <f>E13/C13</f>
+        <v>300</v>
+      </c>
+      <c r="E13">
+        <v>3000</v>
+      </c>
+      <c r="F13">
+        <f t="shared" ref="F13:F20" si="4">IF(ISBLANK(B13), "", VLOOKUP(B13,$O$24:$P$32, 2, FALSE))</f>
+        <v>0.1</v>
+      </c>
+      <c r="G13">
+        <v>0.2</v>
+      </c>
+      <c r="H13">
+        <f t="shared" ref="H13" si="5">D13*IF(G13&lt;&gt;"", G13, F13)</f>
+        <v>60</v>
+      </c>
+      <c r="J13">
+        <f>IF(ISBLANK(B13), "", IF(ISNUMBER(G13), G13*E13, F13*E13))</f>
+        <v>600</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="3"/>
+        <v>5.2810000000000001E-3</v>
+      </c>
+      <c r="L13">
+        <f>IF(ISBLANK(K13), "",$P$4)</f>
+        <v>1.57</v>
+      </c>
+      <c r="M13">
+        <f>IF(ISBLANK(A13), "", J13*K13*L13/1000)</f>
+        <v>4.974702000000001E-3</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="P13" s="2">
         <v>5.3E-3</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" ht="34">
+      <c r="R13" s="2"/>
+    </row>
+    <row r="14" spans="1:18" ht="34">
       <c r="A14" s="3" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C14" s="2">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="D14">
-        <f t="shared" ref="D14:D23" si="5">E14/C14</f>
-        <v>50</v>
+        <f>E14/C14</f>
+        <v>500</v>
       </c>
       <c r="E14">
         <v>5000</v>
       </c>
       <c r="F14">
-        <f>IF(ISBLANK(B14), "", VLOOKUP(B14,$O$24:$P$30, 2, FALSE))</f>
+        <f t="shared" si="4"/>
         <v>0.33700000000000002</v>
       </c>
+      <c r="H14">
+        <f t="shared" ref="H14:H19" si="6">D14*IF(G14&lt;&gt;"", G14, F14)</f>
+        <v>168.5</v>
+      </c>
       <c r="J14">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B14), "", IF(ISNUMBER(G14), G14*E14, F14*E14))</f>
         <v>1685</v>
       </c>
       <c r="K14">
-        <f>(0.0781 + (0.0075*D14)) * 10^-2</f>
-        <v>4.5310000000000003E-3</v>
+        <f t="shared" si="3"/>
+        <v>1.34185E-2</v>
       </c>
       <c r="L14">
         <f>IF(ISBLANK(K14), "",$P$4)</f>
@@ -1360,47 +1435,51 @@
       </c>
       <c r="M14">
         <f>IF(ISBLANK(A14), "", J14*K14*L14/1000)</f>
-        <v>1.1986533950000001E-2</v>
+        <v>3.5497970825000003E-2</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="P14" s="2">
         <v>6.4000000000000003E-3</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" ht="34">
+      <c r="R14" s="2"/>
+    </row>
+    <row r="15" spans="1:18" ht="34">
       <c r="A15" s="3" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C15" s="2">
-        <f>3000 / 20</f>
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="D15">
-        <f t="shared" si="5"/>
-        <v>20</v>
+        <f>E15/C15</f>
+        <v>300</v>
       </c>
       <c r="E15">
         <v>3000</v>
       </c>
       <c r="F15">
-        <f>IF(ISBLANK(B15), "", VLOOKUP(B15,$O$24:$P$30, 2, FALSE))</f>
+        <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
       <c r="G15">
         <v>0.2</v>
       </c>
+      <c r="H15">
+        <f t="shared" si="6"/>
+        <v>60</v>
+      </c>
       <c r="J15">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B15), "", IF(ISNUMBER(G15), G15*E15, F15*E15))</f>
         <v>600</v>
       </c>
       <c r="K15">
-        <f>(0.0781 + (0.0075*D15)) * 10^-2</f>
-        <v>2.281E-3</v>
+        <f t="shared" si="3"/>
+        <v>5.2810000000000001E-3</v>
       </c>
       <c r="L15">
         <f>IF(ISBLANK(K15), "",$P$4)</f>
@@ -1408,95 +1487,206 @@
       </c>
       <c r="M15">
         <f>IF(ISBLANK(A15), "", J15*K15*L15/1000)</f>
-        <v>2.1487020000000002E-3</v>
+        <v>4.974702000000001E-3</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="P15" s="2">
         <v>2.5999999999999999E-3</v>
       </c>
-    </row>
-    <row r="16" spans="1:16">
-      <c r="J16" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="R15" s="2"/>
+    </row>
+    <row r="16" spans="1:18" ht="17">
+      <c r="A16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="2">
+        <v>10</v>
+      </c>
+      <c r="D16">
+        <f>E16/C16</f>
+        <v>30</v>
+      </c>
+      <c r="E16">
+        <v>300</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="4"/>
+        <v>0.27</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="6"/>
+        <v>8.1000000000000014</v>
+      </c>
+      <c r="J16">
+        <f>IF(ISBLANK(B16), "", IF(ISNUMBER(G16), G16*E16, F16*E16))</f>
+        <v>81</v>
+      </c>
+      <c r="K16">
+        <f t="shared" si="3"/>
+        <v>2.9030199720675299E-3</v>
+      </c>
+      <c r="L16">
+        <f>IF(ISBLANK(K16), "",$P$4)</f>
+        <v>1.57</v>
+      </c>
+      <c r="M16">
+        <f>IF(ISBLANK(A16), "", J16*K16*L16/1000)</f>
+        <v>3.6917704984782779E-4</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="P16" s="2">
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:16">
-      <c r="F17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="L17" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="M17" t="str">
+    <row r="17" spans="1:16" ht="17">
+      <c r="A17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="2">
+        <v>10</v>
+      </c>
+      <c r="D17">
+        <f t="shared" ref="D17:D21" si="7">E17/C17</f>
+        <v>35</v>
+      </c>
+      <c r="E17">
+        <v>350</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="4"/>
+        <v>0.33700000000000002</v>
+      </c>
+      <c r="G17">
+        <v>0.5</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="6"/>
+        <v>17.5</v>
+      </c>
+      <c r="J17">
+        <f>IF(ISBLANK(B17), "", IF(ISNUMBER(G17), G17*E17, F17*E17))</f>
+        <v>175</v>
+      </c>
+      <c r="K17">
         <f t="shared" si="3"/>
-        <v/>
+        <v>2.9036430318320843E-3</v>
+      </c>
+      <c r="L17">
+        <f>IF(ISBLANK(K17), "",$P$4)</f>
+        <v>1.57</v>
+      </c>
+      <c r="M17">
+        <f>IF(ISBLANK(A17), "", J17*K17*L17/1000)</f>
+        <v>7.977759229958652E-4</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="P17" s="2">
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:16">
-      <c r="F18" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" t="s">
-        <v>53</v>
+    <row r="18" spans="1:16" ht="17">
+      <c r="A18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="2">
+        <v>10</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="7"/>
+        <v>670</v>
+      </c>
+      <c r="E18">
+        <v>6700</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="4"/>
+        <v>0.46</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="6"/>
+        <v>308.2</v>
+      </c>
+      <c r="J18">
+        <f t="shared" ref="J18:J19" si="8">IF(ISBLANK(B18), "", IF(ISNUMBER(G18), G18*E18, F18*E18))</f>
+        <v>3082</v>
+      </c>
+      <c r="K18">
+        <f>MAX(_xlfn.IFS(A18="Irrigated crop (maize)", (-0.1474 + (0.0061 * H18)) * 10^-2, A18="Non-irrigated crop (high rainfall)", (0.0781 + (0.0075*H18)) * 10^-2, A18="Cotton", ((0.29 + (0.007*(EXP(0.037*MIN(H18, 300)) - 1)/MIN(H18, 300))) * 10^-2)), 0)</f>
+        <v>1.8339704039287866E-2</v>
       </c>
       <c r="L18">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(K18), "",$P$4)</f>
         <v>1.57</v>
       </c>
-      <c r="M18" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="M18">
+        <f>IF(ISBLANK(A18), "", J18*K18*L18/1000)</f>
+        <v>8.8741059523063784E-2</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="P18" s="2">
         <v>2.5999999999999999E-3</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="17">
-      <c r="A19" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" t="s">
-        <v>52</v>
+      <c r="A19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="2">
+        <v>10</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="7"/>
+        <v>200</v>
+      </c>
+      <c r="E19">
+        <v>2000</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="4"/>
+        <v>0.33700000000000002</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="6"/>
+        <v>67.400000000000006</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="8"/>
+        <v>674</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="3"/>
+        <v>2.9115356636702783E-3</v>
+      </c>
+      <c r="L19">
+        <f>IF(ISBLANK(K19), "",$P$4)</f>
+        <v>1.57</v>
+      </c>
+      <c r="M19">
+        <f>IF(ISBLANK(A19), "", J19*K19*L19/1000)</f>
+        <v>3.0809288085826151E-3</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="P19" s="2">
         <v>1.8E-3</v>
@@ -1504,33 +1694,36 @@
     </row>
     <row r="20" spans="1:16" ht="17">
       <c r="A20" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="C20" s="2">
-        <f>300 / 20</f>
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D20">
-        <f t="shared" si="5"/>
-        <v>20</v>
+        <f t="shared" si="7"/>
+        <v>600</v>
       </c>
       <c r="E20">
-        <v>300</v>
+        <v>6000</v>
       </c>
       <c r="F20">
-        <f>IF(ISBLANK(B20), "", VLOOKUP(B20,$O$24:$P$30, 2, FALSE))</f>
-        <v>0.27</v>
+        <f t="shared" si="4"/>
+        <v>0.21</v>
+      </c>
+      <c r="H20">
+        <f t="shared" ref="H20:H21" si="9">D20*IF(G20&lt;&gt;"", G20, F20)</f>
+        <v>126</v>
       </c>
       <c r="J20">
-        <f t="shared" si="1"/>
-        <v>81</v>
+        <f t="shared" ref="J20:J21" si="10">IF(ISBLANK(B20), "", IF(ISNUMBER(G20), G20*E20, F20*E20))</f>
+        <v>1260</v>
       </c>
       <c r="K20">
-        <f>MIN(((0.29 + (0.007*(EXP(0.037*D20) - 1)/D20)) * 10^-2), 0.0183)</f>
-        <v>2.9038357743007299E-3</v>
+        <f t="shared" ref="K20:K21" si="11">MAX(_xlfn.IFS(A20="Irrigated crop (maize)", (-0.1474 + (0.0061 * H20)) * 10^-2, A20="Non-irrigated crop (high rainfall)", (0.0781 + (0.0075*H20)) * 10^-2, A20="Cotton", ((0.29 + (0.007*(EXP(0.037*MIN(H20, 300)) - 1)/MIN(H20, 300))) * 10^-2)), 0)</f>
+        <v>2.9582486476300309E-3</v>
       </c>
       <c r="L20">
         <f>IF(ISBLANK(K20), "",$P$4)</f>
@@ -1538,41 +1731,41 @@
       </c>
       <c r="M20">
         <f>IF(ISBLANK(A20), "", J20*K20*L20/1000)</f>
-        <v>3.6928079541782383E-4</v>
+        <v>5.852007474741727E-3</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="17">
       <c r="A21" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="C21" s="2">
-        <f>350/25</f>
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D21">
-        <f t="shared" si="5"/>
-        <v>25</v>
+        <f t="shared" si="7"/>
+        <v>500</v>
       </c>
       <c r="E21">
-        <v>350</v>
+        <v>5000</v>
       </c>
       <c r="F21">
-        <f>IF(ISBLANK(B21), "", VLOOKUP(B21,$O$24:$P$30, 2, FALSE))</f>
-        <v>0.33700000000000002</v>
-      </c>
-      <c r="G21">
-        <v>0.5</v>
+        <f t="shared" ref="F21" si="12">IF(ISBLANK(B21), "", VLOOKUP(B21,$O$24:$P$32, 2, FALSE))</f>
+        <v>0.155</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="9"/>
+        <v>77.5</v>
       </c>
       <c r="J21">
-        <f t="shared" si="1"/>
-        <v>175</v>
+        <f t="shared" si="10"/>
+        <v>775</v>
       </c>
       <c r="K21">
-        <f>MIN(((0.29 + (0.007*(EXP(0.037*D21) - 1)/D21)) * 10^-2), 0.0183)</f>
-        <v>2.9042612311290027E-3</v>
+        <f t="shared" si="11"/>
+        <v>2.914987208395978E-3</v>
       </c>
       <c r="L21">
         <f>IF(ISBLANK(K21), "",$P$4)</f>
@@ -1580,112 +1773,27 @@
       </c>
       <c r="M21">
         <f>IF(ISBLANK(A21), "", J21*K21*L21/1000)</f>
-        <v>7.9794577325269353E-4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" ht="17">
-      <c r="A22" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C22" s="2">
-        <v>800</v>
-      </c>
-      <c r="D22">
-        <f t="shared" si="5"/>
-        <v>27.75</v>
-      </c>
-      <c r="E22">
-        <v>22200</v>
-      </c>
-      <c r="F22">
-        <f>IF(ISBLANK(B22), "", VLOOKUP(B22,$O$24:$P$30, 2, FALSE))</f>
-        <v>0.46</v>
-      </c>
-      <c r="J22">
-        <f t="shared" ref="J22" si="6">IF(ISBLANK(B22), "", IF(ISNUMBER(G22), G22*E22, F22*E22))</f>
-        <v>10212</v>
-      </c>
-      <c r="K22">
-        <f>MIN(((0.29 + (0.007*(EXP(0.037*D22) - 1)/D22)) * 10^-2), 0.0183)</f>
-        <v>2.9045203027153032E-3</v>
-      </c>
-      <c r="L22">
-        <f>IF(ISBLANK(K22), "",$P$4)</f>
-        <v>1.57</v>
-      </c>
-      <c r="M22">
-        <f>IF(ISBLANK(A22), "", J22*K22*L22/1000)</f>
-        <v>4.6567709290186027E-2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" ht="17">
-      <c r="A23" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="2">
-        <f>22300/25</f>
-        <v>892</v>
-      </c>
-      <c r="D23">
-        <f t="shared" si="5"/>
-        <v>25</v>
-      </c>
-      <c r="E23">
-        <v>22300</v>
-      </c>
-      <c r="F23">
-        <f>IF(ISBLANK(B23), "", VLOOKUP(B23,$O$24:$P$30, 2, FALSE))</f>
-        <v>0.33700000000000002</v>
-      </c>
-      <c r="J23">
-        <f t="shared" ref="J23" si="7">IF(ISBLANK(B23), "", IF(ISNUMBER(G23), G23*E23, F23*E23))</f>
-        <v>7515.1</v>
-      </c>
-      <c r="K23">
-        <f>MIN(((0.29 + (0.007*(EXP(0.037*D23) - 1)/D23)) * 10^-2), 0.0183)</f>
-        <v>2.9042612311290027E-3</v>
-      </c>
-      <c r="L23">
-        <f>IF(ISBLANK(K23), "",$P$4)</f>
-        <v>1.57</v>
-      </c>
-      <c r="M23">
-        <f>IF(ISBLANK(A23), "", J23*K23*L23/1000)</f>
-        <v>3.4266527317550387E-2</v>
-      </c>
-      <c r="O23" s="2" t="s">
-        <v>11</v>
+        <v>3.5468106858158066E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16">
+      <c r="O23" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:16">
-      <c r="H24" t="str">
-        <f t="shared" ref="H24:H25" si="8">IF(ISBLANK(D24), "", E24/D24)</f>
-        <v/>
-      </c>
-      <c r="J24" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="A24" s="4"/>
+      <c r="K24" s="1"/>
       <c r="O24" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="P24" s="2">
         <v>0.1</v>
       </c>
     </row>
     <row r="25" spans="1:16">
-      <c r="H25" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
       <c r="O25" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="P25" s="2">
         <v>0.18</v>
@@ -1693,42 +1801,105 @@
     </row>
     <row r="26" spans="1:16">
       <c r="O26" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="P26" s="2">
         <v>0.46</v>
       </c>
     </row>
     <row r="27" spans="1:16">
+      <c r="J27" t="str">
+        <f>IF(ISBLANK(B27), "", IF(ISNUMBER(G27), G27*E27, F27*E27))</f>
+        <v/>
+      </c>
       <c r="O27" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="P27" s="2">
         <v>0.21</v>
       </c>
     </row>
     <row r="28" spans="1:16">
+      <c r="F28" t="str">
+        <f>IF(ISBLANK(B28), "", VLOOKUP(B28,$O$24:$P$30, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <f>IF(ISBLANK(B28), "", IF(ISNUMBER(G28), G28*E28, F28*E28))</f>
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <f>IF(ISBLANK(K28), "",$P$4)</f>
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <f>IF(ISBLANK(A28), "", J28*K28*L28/1000)</f>
+        <v/>
+      </c>
       <c r="O28" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P28" s="2">
         <v>0.32</v>
       </c>
     </row>
     <row r="29" spans="1:16">
+      <c r="F29" t="str">
+        <f>IF(ISBLANK(B29), "", VLOOKUP(B29,$O$24:$P$30, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <f>IF(ISBLANK(B29), "", IF(ISNUMBER(G29), G29*E29, F29*E29))</f>
+        <v/>
+      </c>
+      <c r="L29" t="str">
+        <f>IF(ISBLANK(K29), "",$P$4)</f>
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <f>IF(ISBLANK(A29), "", J29*K29*L29/1000)</f>
+        <v/>
+      </c>
       <c r="O29" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="P29" s="2">
         <v>0.33700000000000002</v>
       </c>
     </row>
     <row r="30" spans="1:16">
+      <c r="A30" s="4"/>
       <c r="O30" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="P30" s="2">
         <v>0.27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16">
+      <c r="O31" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="P31">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16">
+      <c r="O32" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="P32">
+        <v>0.155</v>
+      </c>
+    </row>
+    <row r="35" spans="8:10">
+      <c r="H35" t="str">
+        <f>IF(ISBLANK(D35), "", E35/D35)</f>
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <f>IF(ISBLANK(B35), "", IF(ISNUMBER(G35), G35*E35, F35*E35))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1750,13 +1921,13 @@
   <sheetData>
     <row r="1" spans="1:15" ht="17">
       <c r="A1" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -1771,51 +1942,51 @@
       <c r="I4" s="1"/>
       <c r="L4" s="1"/>
       <c r="N4" s="9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="D5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I5" s="1"/>
       <c r="L5" s="1"/>
     </row>
     <row r="6" spans="1:15" ht="17">
       <c r="A6" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>5</v>
       </c>
       <c r="H6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="J6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="17">
       <c r="A7" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C7">
         <v>100</v>
@@ -1844,7 +2015,7 @@
         <v>3.6700000000000003E-2</v>
       </c>
       <c r="N7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="O7">
         <f>[1]!common_cco2</f>
@@ -1853,10 +2024,10 @@
     </row>
     <row r="8" spans="1:15" ht="17">
       <c r="A8" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C8">
         <v>100</v>
@@ -1887,10 +2058,10 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C9">
         <v>100</v>
@@ -1919,7 +2090,7 @@
         <v>0</v>
       </c>
       <c r="N9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="O9">
         <v>0.2</v>
@@ -2051,7 +2222,7 @@
         <v/>
       </c>
       <c r="N26" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="2:15">
@@ -2064,7 +2235,7 @@
         <v/>
       </c>
       <c r="N27" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="O27" s="2">
         <v>0</v>
@@ -2076,7 +2247,7 @@
         <v/>
       </c>
       <c r="N28" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="O28" s="2">
         <v>0</v>
@@ -2084,7 +2255,7 @@
     </row>
     <row r="29" spans="2:15">
       <c r="N29" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="O29" s="2">
         <v>1</v>
@@ -2092,7 +2263,7 @@
     </row>
     <row r="30" spans="2:15">
       <c r="N30" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O30" s="2">
         <v>0</v>
@@ -2100,7 +2271,7 @@
     </row>
     <row r="31" spans="2:15">
       <c r="N31" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="O31" s="2">
         <v>0.35</v>
@@ -2108,7 +2279,7 @@
     </row>
     <row r="32" spans="2:15">
       <c r="N32" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="O32" s="2">
         <v>0</v>
@@ -2116,7 +2287,7 @@
     </row>
     <row r="33" spans="14:15">
       <c r="N33" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O33" s="2">
         <v>0</v>

</xml_diff>